<commit_message>
add songs to list, fix 2024 fra
</commit_message>
<xml_diff>
--- a/data/repository/raw_data.xlsx
+++ b/data/repository/raw_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vu00388\git\ultrastar2singIt\data\repository\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\anton\git\ultrastar2singIt\data\repository\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8CD9D14-AFAD-4873-B5FA-C28776A67B0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E678BB8-27C1-4465-835A-B28E3BD703F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{97B7E96E-B014-403A-BA4F-9DB5B3CEF783}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{97B7E96E-B014-403A-BA4F-9DB5B3CEF783}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,8 +27,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -36,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="145">
   <si>
     <t>0100CC30149B900D</t>
   </si>
@@ -303,13 +301,181 @@
   </si>
   <si>
     <t>core_edition</t>
+  </si>
+  <si>
+    <t>songs_fra</t>
+  </si>
+  <si>
+    <t>0100953009DF9002</t>
+  </si>
+  <si>
+    <t>0100953009DF9007</t>
+  </si>
+  <si>
+    <t>0100953009DF9006</t>
+  </si>
+  <si>
+    <t>0100953009DF9003</t>
+  </si>
+  <si>
+    <t>0100953009DF9005</t>
+  </si>
+  <si>
+    <t>0100953009DF9001</t>
+  </si>
+  <si>
+    <t>0100953009DF9004</t>
+  </si>
+  <si>
+    <t>010065F00DF4B007</t>
+  </si>
+  <si>
+    <t>010065F00DF4B002</t>
+  </si>
+  <si>
+    <t>010065F00DF4B006</t>
+  </si>
+  <si>
+    <t>010065F00DF4B008</t>
+  </si>
+  <si>
+    <t>010065F00DF4B003</t>
+  </si>
+  <si>
+    <t>010065F00DF4B009</t>
+  </si>
+  <si>
+    <t>010065F00DF4B005</t>
+  </si>
+  <si>
+    <t>010065F00DF4B001</t>
+  </si>
+  <si>
+    <t>010065F00DF4B004</t>
+  </si>
+  <si>
+    <t>010061F0119FB002</t>
+  </si>
+  <si>
+    <t>010061F0119FB007</t>
+  </si>
+  <si>
+    <t>010061F0119FB00A</t>
+  </si>
+  <si>
+    <t>010061F0119FB006</t>
+  </si>
+  <si>
+    <t>010061F0119FB008</t>
+  </si>
+  <si>
+    <t>010061F0119FB003</t>
+  </si>
+  <si>
+    <t>010061F0119FB00B</t>
+  </si>
+  <si>
+    <t>010061F0119FB009</t>
+  </si>
+  <si>
+    <t>010061F0119FB005</t>
+  </si>
+  <si>
+    <t>010061F0119FB001</t>
+  </si>
+  <si>
+    <t>010061F0119FB004</t>
+  </si>
+  <si>
+    <t>0100382004207002</t>
+  </si>
+  <si>
+    <t>0100382004207003</t>
+  </si>
+  <si>
+    <t>0100382004207005</t>
+  </si>
+  <si>
+    <t>0100382004207001</t>
+  </si>
+  <si>
+    <t>0100382004207004</t>
+  </si>
+  <si>
+    <t>DLC Best of 80's Song Pack</t>
+  </si>
+  <si>
+    <t>DLC Chart Hits Song Pack</t>
+  </si>
+  <si>
+    <t>DLC Legendary Hits Song Pack</t>
+  </si>
+  <si>
+    <t>DLC Party Classics Song Pack</t>
+  </si>
+  <si>
+    <t>DLC Party Classics Vol 2 Song Pack</t>
+  </si>
+  <si>
+    <t>DLC Best of 80's Vol 1 Song Pack</t>
+  </si>
+  <si>
+    <t>DLC Best of 80's Vol 2 Song Pack</t>
+  </si>
+  <si>
+    <t>DLC Best of 90's Song Pack</t>
+  </si>
+  <si>
+    <t>DLC Party Classics Vol 1 Song Pack</t>
+  </si>
+  <si>
+    <t>DLC Best of 80's Vol. 1 Song Pack</t>
+  </si>
+  <si>
+    <t>DLC Best of 90's Vol 1 Song Pack</t>
+  </si>
+  <si>
+    <t>DLC Best of 90's Vol 2 Song Pack</t>
+  </si>
+  <si>
+    <t>DLC Country Hits Song Pack</t>
+  </si>
+  <si>
+    <t>DLC Best of 80s Vol 1 Song Pack</t>
+  </si>
+  <si>
+    <t>DLC Best of 80s Vol 2 Song Pack</t>
+  </si>
+  <si>
+    <t>DLC Best of 80s Vol 3 Song Pack</t>
+  </si>
+  <si>
+    <t>DLC Best of 90s Vol 1 Song Pack</t>
+  </si>
+  <si>
+    <t>DLC Best of 90s Vol 2 Song Pack</t>
+  </si>
+  <si>
+    <t>DLC Classic Rock Song Pack</t>
+  </si>
+  <si>
+    <t>0100953009DF8000</t>
+  </si>
+  <si>
+    <t>010065F00DF4A000</t>
+  </si>
+  <si>
+    <t>010061F0119FA000</t>
+  </si>
+  <si>
+    <t>0100382004206000</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -346,8 +512,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -682,19 +849,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD1735EA-D059-4AAA-91E6-6B0DCE3BA57A}">
-  <dimension ref="A1:E41"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:E72"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="18" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.75" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:5">
+      <c r="A1" s="1" t="s">
         <v>34</v>
       </c>
       <c r="B1" t="s">
@@ -703,580 +870,1023 @@
       <c r="C1" t="s">
         <v>87</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>35</v>
       </c>
       <c r="E1" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="2" spans="1:5">
+      <c r="A2" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="B2" t="s">
+        <v>122</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="E2">
+        <v>2018</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="B3" t="s">
+        <v>123</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="E3">
+        <v>2018</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="B4" t="s">
+        <v>124</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="E4">
+        <v>2018</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="B5" t="s">
+        <v>125</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="E5">
+        <v>2018</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="B6" t="s">
+        <v>126</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="E6">
+        <v>2018</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B7" t="s">
+        <v>127</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="E7">
+        <v>2019</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
+      <c r="A8" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="B8" t="s">
+        <v>128</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="E8">
+        <v>2019</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
+      <c r="A9" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="B9" t="s">
+        <v>129</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="E9">
+        <v>2019</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="A10" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B10" t="s">
+        <v>123</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="E10">
+        <v>2019</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
+      <c r="A11" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="B11" t="s">
+        <v>124</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="E11">
+        <v>2019</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
+      <c r="A12" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B12" t="s">
+        <v>130</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="E12">
+        <v>2019</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
+      <c r="A13" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B13" t="s">
+        <v>126</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="E13">
+        <v>2019</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5">
+      <c r="A14" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="B14" t="s">
+        <v>128</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="E14">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5">
+      <c r="A15" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="B15" t="s">
+        <v>131</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="E15">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5">
+      <c r="A16" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="B16" t="s">
+        <v>132</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="E16">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5">
+      <c r="A17" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="B17" t="s">
+        <v>133</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="E17">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5">
+      <c r="A18" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="B18" t="s">
+        <v>123</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="E18">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5">
+      <c r="A19" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="B19" t="s">
+        <v>134</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="E19">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5">
+      <c r="A20" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="B20" t="s">
+        <v>124</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="E20">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5">
+      <c r="A21" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B21" t="s">
+        <v>130</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="E21">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5">
+      <c r="A22" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="B22" t="s">
+        <v>126</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="E22">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5">
+      <c r="A23" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="B23" t="s">
+        <v>135</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="E23">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5">
+      <c r="A24" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="B24" t="s">
+        <v>136</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="E24">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5">
+      <c r="A25" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="B25" t="s">
+        <v>137</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="E25">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5">
+      <c r="A26" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="B26" t="s">
+        <v>138</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="E26">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5">
+      <c r="A27" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="B27" t="s">
+        <v>139</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="E27">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5">
+      <c r="A28" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="B28" t="s">
+        <v>123</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="E28">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5">
+      <c r="A29" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="B29" t="s">
+        <v>140</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="E29">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5">
+      <c r="A30" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="B30" t="s">
+        <v>134</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="E30">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5">
+      <c r="A31" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="B31" t="s">
+        <v>124</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="E31">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5">
+      <c r="A32" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="B32" t="s">
+        <v>130</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="E32">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5">
+      <c r="A33" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="B33" t="s">
+        <v>126</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="E33">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5">
+      <c r="A34" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B34" t="s">
         <v>8</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D34" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="E2">
+      <c r="E34">
         <v>2022</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="35" spans="1:5">
+      <c r="A35" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B35" t="s">
         <v>9</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D35" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="E3">
+      <c r="E35">
         <v>2022</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row r="36" spans="1:5">
+      <c r="A36" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B36" t="s">
         <v>10</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D36" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="E4">
+      <c r="E36">
         <v>2022</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+    <row r="37" spans="1:5">
+      <c r="A37" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B37" t="s">
         <v>11</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D37" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="E5">
+      <c r="E37">
         <v>2022</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+    <row r="38" spans="1:5">
+      <c r="A38" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B38" t="s">
         <v>12</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D38" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="E6">
+      <c r="E38">
         <v>2022</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+    <row r="39" spans="1:5">
+      <c r="A39" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B39" t="s">
         <v>13</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D39" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="E7">
+      <c r="E39">
         <v>2022</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+    <row r="40" spans="1:5">
+      <c r="A40" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B40" t="s">
         <v>14</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D40" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="E8">
+      <c r="E40">
         <v>2022</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+    <row r="41" spans="1:5">
+      <c r="A41" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B41" t="s">
         <v>15</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D41" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="E9">
+      <c r="E41">
         <v>2022</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+    <row r="42" spans="1:5">
+      <c r="A42" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B42" t="s">
         <v>16</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D42" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="E10">
+      <c r="E42">
         <v>2022</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+    <row r="43" spans="1:5">
+      <c r="A43" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B43" t="s">
         <v>17</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D43" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="E11">
+      <c r="E43">
         <v>2022</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+    <row r="44" spans="1:5">
+      <c r="A44" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B44" t="s">
         <v>18</v>
       </c>
-      <c r="D12" t="s">
+      <c r="D44" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="E12">
+      <c r="E44">
         <v>2022</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+    <row r="45" spans="1:5">
+      <c r="A45" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B45" t="s">
         <v>19</v>
       </c>
-      <c r="D13" t="s">
+      <c r="D45" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="E13">
+      <c r="E45">
         <v>2022</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+    <row r="46" spans="1:5">
+      <c r="A46" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B46" t="s">
         <v>20</v>
       </c>
-      <c r="D14" t="s">
+      <c r="D46" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="E14">
+      <c r="E46">
         <v>2022</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
+    <row r="47" spans="1:5">
+      <c r="A47" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B47" t="s">
         <v>21</v>
       </c>
-      <c r="D15" t="s">
+      <c r="D47" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="E15">
+      <c r="E47">
         <v>2022</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+    <row r="48" spans="1:5">
+      <c r="A48" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B48" t="s">
         <v>22</v>
       </c>
-      <c r="D16" t="s">
+      <c r="D48" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="E16">
+      <c r="E48">
         <v>2022</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
+    <row r="49" spans="1:5">
+      <c r="A49" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B49" t="s">
         <v>23</v>
       </c>
-      <c r="D17" t="s">
+      <c r="D49" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="E17">
+      <c r="E49">
         <v>2022</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
+    <row r="50" spans="1:5">
+      <c r="A50" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B50" t="s">
         <v>24</v>
       </c>
-      <c r="D18" t="s">
+      <c r="D50" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="E18">
+      <c r="E50">
         <v>2022</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
+    <row r="51" spans="1:5">
+      <c r="A51" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B51" t="s">
         <v>55</v>
       </c>
-      <c r="D19" t="s">
+      <c r="D51" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="E19">
+      <c r="E51">
         <v>2023</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
+    <row r="52" spans="1:5">
+      <c r="A52" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B52" t="s">
         <v>56</v>
       </c>
-      <c r="D20" t="s">
+      <c r="D52" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="E20">
+      <c r="E52">
         <v>2023</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
+    <row r="53" spans="1:5">
+      <c r="A53" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B53" t="s">
         <v>57</v>
       </c>
-      <c r="D21" t="s">
+      <c r="D53" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="E21">
+      <c r="E53">
         <v>2023</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
+    <row r="54" spans="1:5">
+      <c r="A54" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B54" t="s">
         <v>58</v>
       </c>
-      <c r="D22" t="s">
+      <c r="D54" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="E22">
+      <c r="E54">
         <v>2023</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
+    <row r="55" spans="1:5">
+      <c r="A55" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B55" t="s">
         <v>59</v>
       </c>
-      <c r="D23" t="s">
+      <c r="D55" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="E23">
+      <c r="E55">
         <v>2023</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
+    <row r="56" spans="1:5">
+      <c r="A56" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B56" t="s">
         <v>60</v>
       </c>
-      <c r="D24" t="s">
+      <c r="D56" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="E24">
+      <c r="E56">
         <v>2023</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
+    <row r="57" spans="1:5">
+      <c r="A57" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B57" t="s">
         <v>14</v>
       </c>
-      <c r="D25" t="s">
+      <c r="D57" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="E25">
+      <c r="E57">
         <v>2023</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
+    <row r="58" spans="1:5">
+      <c r="A58" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B58" t="s">
         <v>61</v>
       </c>
-      <c r="D26" t="s">
+      <c r="D58" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="E26">
+      <c r="E58">
         <v>2023</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
+    <row r="59" spans="1:5">
+      <c r="A59" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="B27" t="s">
+      <c r="B59" t="s">
         <v>15</v>
       </c>
-      <c r="D27" t="s">
+      <c r="D59" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="E27">
+      <c r="E59">
         <v>2023</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
+    <row r="60" spans="1:5">
+      <c r="A60" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B28" t="s">
+      <c r="B60" t="s">
         <v>16</v>
       </c>
-      <c r="D28" t="s">
+      <c r="D60" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="E28">
+      <c r="E60">
         <v>2023</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
+    <row r="61" spans="1:5">
+      <c r="A61" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="B29" t="s">
+      <c r="B61" t="s">
         <v>62</v>
       </c>
-      <c r="D29" t="s">
+      <c r="D61" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="E29">
+      <c r="E61">
         <v>2023</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
+    <row r="62" spans="1:5">
+      <c r="A62" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="B30" t="s">
+      <c r="B62" t="s">
         <v>63</v>
       </c>
-      <c r="D30" t="s">
+      <c r="D62" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="E30">
+      <c r="E62">
         <v>2023</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
+    <row r="63" spans="1:5">
+      <c r="A63" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="B31" t="s">
+      <c r="B63" t="s">
         <v>64</v>
       </c>
-      <c r="D31" t="s">
+      <c r="D63" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="E31">
+      <c r="E63">
         <v>2023</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
+    <row r="64" spans="1:5">
+      <c r="A64" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="B32" t="s">
+      <c r="B64" t="s">
         <v>65</v>
       </c>
-      <c r="D32" t="s">
+      <c r="D64" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="E32">
+      <c r="E64">
         <v>2023</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
+    <row r="65" spans="1:5">
+      <c r="A65" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B33" t="s">
+      <c r="B65" t="s">
         <v>66</v>
       </c>
-      <c r="D33" t="s">
+      <c r="D65" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="E33">
+      <c r="E65">
         <v>2023</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
+    <row r="66" spans="1:5">
+      <c r="A66" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="B34" t="s">
+      <c r="B66" t="s">
         <v>67</v>
       </c>
-      <c r="D34" t="s">
+      <c r="D66" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="E34">
+      <c r="E66">
         <v>2023</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
+    <row r="67" spans="1:5">
+      <c r="A67" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="B35" t="s">
+      <c r="B67" t="s">
         <v>74</v>
       </c>
-      <c r="C35" t="s">
+      <c r="C67" t="s">
         <v>82</v>
       </c>
-      <c r="D35" t="s">
+      <c r="D67" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="E35">
+      <c r="E67">
         <v>2024</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
+    <row r="68" spans="1:5">
+      <c r="A68" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B36" t="s">
+      <c r="B68" t="s">
         <v>75</v>
       </c>
-      <c r="C36" t="s">
+      <c r="C68" t="s">
         <v>81</v>
       </c>
-      <c r="D36" t="s">
+      <c r="D68" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="E36">
+      <c r="E68">
         <v>2024</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
+    <row r="69" spans="1:5">
+      <c r="A69" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="B37" t="s">
+      <c r="B69" t="s">
         <v>76</v>
       </c>
-      <c r="C37" t="s">
+      <c r="C69" t="s">
+        <v>89</v>
+      </c>
+      <c r="D69" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E69">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5">
+      <c r="A70" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B70" t="s">
+        <v>77</v>
+      </c>
+      <c r="C70" t="s">
+        <v>80</v>
+      </c>
+      <c r="D70" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E70">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5">
+      <c r="A71" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="B71" t="s">
+        <v>78</v>
+      </c>
+      <c r="C71" t="s">
+        <v>79</v>
+      </c>
+      <c r="D71" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E71">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5">
+      <c r="A72" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="B72" t="s">
+        <v>84</v>
+      </c>
+      <c r="C72" t="s">
         <v>85</v>
       </c>
-      <c r="D37" t="s">
-        <v>68</v>
-      </c>
-      <c r="E37">
-        <v>2024</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>72</v>
-      </c>
-      <c r="B38" t="s">
-        <v>77</v>
-      </c>
-      <c r="C38" t="s">
-        <v>80</v>
-      </c>
-      <c r="D38" t="s">
-        <v>68</v>
-      </c>
-      <c r="E38">
-        <v>2024</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
-        <v>73</v>
-      </c>
-      <c r="B39" t="s">
-        <v>78</v>
-      </c>
-      <c r="C39" t="s">
-        <v>79</v>
-      </c>
-      <c r="D39" t="s">
-        <v>68</v>
-      </c>
-      <c r="E39">
-        <v>2024</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
-        <v>83</v>
-      </c>
-      <c r="B40" t="s">
-        <v>84</v>
-      </c>
-      <c r="C40" t="s">
-        <v>85</v>
-      </c>
-      <c r="D40" t="s">
+      <c r="D72" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="E40">
+      <c r="E72">
         <v>2025</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E41">
-        <v>2026</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add more DLCs to list
</commit_message>
<xml_diff>
--- a/data/repository/raw_data.xlsx
+++ b/data/repository/raw_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\anton\git\ultrastar2singIt\data\repository\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vu00388\git\ultrastar2singIt\data\repository\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E678BB8-27C1-4465-835A-B28E3BD703F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7326876E-1701-4279-B436-C1C08820A8E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{97B7E96E-B014-403A-BA4F-9DB5B3CEF783}"/>
+    <workbookView xWindow="390" yWindow="390" windowWidth="21600" windowHeight="12645" xr2:uid="{97B7E96E-B014-403A-BA4F-9DB5B3CEF783}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="160">
   <si>
     <t>0100CC30149B900D</t>
   </si>
@@ -469,13 +469,58 @@
   </si>
   <si>
     <t>0100382004206000</t>
+  </si>
+  <si>
+    <t>01001C101ED11003</t>
+  </si>
+  <si>
+    <t>German Hits</t>
+  </si>
+  <si>
+    <t>01001C101ED11001</t>
+  </si>
+  <si>
+    <t>Australia and New Zealand Hits</t>
+  </si>
+  <si>
+    <t>01001C101ED11004</t>
+  </si>
+  <si>
+    <t>01001C101ED11005</t>
+  </si>
+  <si>
+    <t>Spanish Hits</t>
+  </si>
+  <si>
+    <t>0100EE4020D18000</t>
+  </si>
+  <si>
+    <t>0100EE4020D19001</t>
+  </si>
+  <si>
+    <t>0100EE4020D19002</t>
+  </si>
+  <si>
+    <t>0100EE4020D19003</t>
+  </si>
+  <si>
+    <t>0100EE4020D19004</t>
+  </si>
+  <si>
+    <t>0100EE4020D19006</t>
+  </si>
+  <si>
+    <t>UK Hits</t>
+  </si>
+  <si>
+    <t>songs_uk</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -849,18 +894,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD1735EA-D059-4AAA-91E6-6B0DCE3BA57A}">
-  <dimension ref="A1:E72"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <dimension ref="A1:E81"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.75" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.85546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>34</v>
       </c>
@@ -877,7 +922,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>117</v>
       </c>
@@ -891,7 +936,7 @@
         <v>2018</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>118</v>
       </c>
@@ -905,7 +950,7 @@
         <v>2018</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>119</v>
       </c>
@@ -919,7 +964,7 @@
         <v>2018</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>120</v>
       </c>
@@ -933,7 +978,7 @@
         <v>2018</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>121</v>
       </c>
@@ -947,7 +992,7 @@
         <v>2018</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>90</v>
       </c>
@@ -961,7 +1006,7 @@
         <v>2019</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>91</v>
       </c>
@@ -975,7 +1020,7 @@
         <v>2019</v>
       </c>
     </row>
-    <row r="9" spans="1:5">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>92</v>
       </c>
@@ -989,7 +1034,7 @@
         <v>2019</v>
       </c>
     </row>
-    <row r="10" spans="1:5">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>93</v>
       </c>
@@ -1003,7 +1048,7 @@
         <v>2019</v>
       </c>
     </row>
-    <row r="11" spans="1:5">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>94</v>
       </c>
@@ -1017,7 +1062,7 @@
         <v>2019</v>
       </c>
     </row>
-    <row r="12" spans="1:5">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>95</v>
       </c>
@@ -1031,7 +1076,7 @@
         <v>2019</v>
       </c>
     </row>
-    <row r="13" spans="1:5">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>96</v>
       </c>
@@ -1045,7 +1090,7 @@
         <v>2019</v>
       </c>
     </row>
-    <row r="14" spans="1:5">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>97</v>
       </c>
@@ -1059,7 +1104,7 @@
         <v>2020</v>
       </c>
     </row>
-    <row r="15" spans="1:5">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>98</v>
       </c>
@@ -1073,7 +1118,7 @@
         <v>2020</v>
       </c>
     </row>
-    <row r="16" spans="1:5">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>99</v>
       </c>
@@ -1087,7 +1132,7 @@
         <v>2020</v>
       </c>
     </row>
-    <row r="17" spans="1:5">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>100</v>
       </c>
@@ -1101,7 +1146,7 @@
         <v>2020</v>
       </c>
     </row>
-    <row r="18" spans="1:5">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>101</v>
       </c>
@@ -1115,7 +1160,7 @@
         <v>2020</v>
       </c>
     </row>
-    <row r="19" spans="1:5">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>102</v>
       </c>
@@ -1129,7 +1174,7 @@
         <v>2020</v>
       </c>
     </row>
-    <row r="20" spans="1:5">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>103</v>
       </c>
@@ -1143,7 +1188,7 @@
         <v>2020</v>
       </c>
     </row>
-    <row r="21" spans="1:5">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>104</v>
       </c>
@@ -1157,7 +1202,7 @@
         <v>2020</v>
       </c>
     </row>
-    <row r="22" spans="1:5">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>105</v>
       </c>
@@ -1171,7 +1216,7 @@
         <v>2020</v>
       </c>
     </row>
-    <row r="23" spans="1:5">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>106</v>
       </c>
@@ -1185,7 +1230,7 @@
         <v>2021</v>
       </c>
     </row>
-    <row r="24" spans="1:5">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>107</v>
       </c>
@@ -1199,7 +1244,7 @@
         <v>2021</v>
       </c>
     </row>
-    <row r="25" spans="1:5">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>108</v>
       </c>
@@ -1213,7 +1258,7 @@
         <v>2021</v>
       </c>
     </row>
-    <row r="26" spans="1:5">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>109</v>
       </c>
@@ -1227,7 +1272,7 @@
         <v>2021</v>
       </c>
     </row>
-    <row r="27" spans="1:5">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>110</v>
       </c>
@@ -1241,7 +1286,7 @@
         <v>2021</v>
       </c>
     </row>
-    <row r="28" spans="1:5">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>111</v>
       </c>
@@ -1255,7 +1300,7 @@
         <v>2021</v>
       </c>
     </row>
-    <row r="29" spans="1:5">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>112</v>
       </c>
@@ -1269,7 +1314,7 @@
         <v>2021</v>
       </c>
     </row>
-    <row r="30" spans="1:5">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>113</v>
       </c>
@@ -1283,7 +1328,7 @@
         <v>2021</v>
       </c>
     </row>
-    <row r="31" spans="1:5">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>114</v>
       </c>
@@ -1297,7 +1342,7 @@
         <v>2021</v>
       </c>
     </row>
-    <row r="32" spans="1:5">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>115</v>
       </c>
@@ -1311,7 +1356,7 @@
         <v>2021</v>
       </c>
     </row>
-    <row r="33" spans="1:5">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>116</v>
       </c>
@@ -1325,7 +1370,7 @@
         <v>2021</v>
       </c>
     </row>
-    <row r="34" spans="1:5">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>25</v>
       </c>
@@ -1339,7 +1384,7 @@
         <v>2022</v>
       </c>
     </row>
-    <row r="35" spans="1:5">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>26</v>
       </c>
@@ -1353,7 +1398,7 @@
         <v>2022</v>
       </c>
     </row>
-    <row r="36" spans="1:5">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>27</v>
       </c>
@@ -1367,7 +1412,7 @@
         <v>2022</v>
       </c>
     </row>
-    <row r="37" spans="1:5">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>28</v>
       </c>
@@ -1381,7 +1426,7 @@
         <v>2022</v>
       </c>
     </row>
-    <row r="38" spans="1:5">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>29</v>
       </c>
@@ -1395,7 +1440,7 @@
         <v>2022</v>
       </c>
     </row>
-    <row r="39" spans="1:5">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>30</v>
       </c>
@@ -1409,7 +1454,7 @@
         <v>2022</v>
       </c>
     </row>
-    <row r="40" spans="1:5">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>31</v>
       </c>
@@ -1423,7 +1468,7 @@
         <v>2022</v>
       </c>
     </row>
-    <row r="41" spans="1:5">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>32</v>
       </c>
@@ -1437,7 +1482,7 @@
         <v>2022</v>
       </c>
     </row>
-    <row r="42" spans="1:5">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>33</v>
       </c>
@@ -1451,7 +1496,7 @@
         <v>2022</v>
       </c>
     </row>
-    <row r="43" spans="1:5">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>0</v>
       </c>
@@ -1465,7 +1510,7 @@
         <v>2022</v>
       </c>
     </row>
-    <row r="44" spans="1:5">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>1</v>
       </c>
@@ -1479,7 +1524,7 @@
         <v>2022</v>
       </c>
     </row>
-    <row r="45" spans="1:5">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
         <v>2</v>
       </c>
@@ -1493,7 +1538,7 @@
         <v>2022</v>
       </c>
     </row>
-    <row r="46" spans="1:5">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>3</v>
       </c>
@@ -1507,7 +1552,7 @@
         <v>2022</v>
       </c>
     </row>
-    <row r="47" spans="1:5">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
         <v>4</v>
       </c>
@@ -1521,7 +1566,7 @@
         <v>2022</v>
       </c>
     </row>
-    <row r="48" spans="1:5">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
         <v>5</v>
       </c>
@@ -1535,7 +1580,7 @@
         <v>2022</v>
       </c>
     </row>
-    <row r="49" spans="1:5">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
         <v>6</v>
       </c>
@@ -1549,7 +1594,7 @@
         <v>2022</v>
       </c>
     </row>
-    <row r="50" spans="1:5">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
         <v>7</v>
       </c>
@@ -1563,7 +1608,7 @@
         <v>2022</v>
       </c>
     </row>
-    <row r="51" spans="1:5">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
         <v>39</v>
       </c>
@@ -1577,7 +1622,7 @@
         <v>2023</v>
       </c>
     </row>
-    <row r="52" spans="1:5">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
         <v>40</v>
       </c>
@@ -1591,7 +1636,7 @@
         <v>2023</v>
       </c>
     </row>
-    <row r="53" spans="1:5">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
         <v>41</v>
       </c>
@@ -1605,7 +1650,7 @@
         <v>2023</v>
       </c>
     </row>
-    <row r="54" spans="1:5">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
         <v>42</v>
       </c>
@@ -1619,7 +1664,7 @@
         <v>2023</v>
       </c>
     </row>
-    <row r="55" spans="1:5">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
         <v>43</v>
       </c>
@@ -1633,7 +1678,7 @@
         <v>2023</v>
       </c>
     </row>
-    <row r="56" spans="1:5">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
         <v>44</v>
       </c>
@@ -1647,7 +1692,7 @@
         <v>2023</v>
       </c>
     </row>
-    <row r="57" spans="1:5">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
         <v>45</v>
       </c>
@@ -1661,7 +1706,7 @@
         <v>2023</v>
       </c>
     </row>
-    <row r="58" spans="1:5">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
         <v>46</v>
       </c>
@@ -1675,7 +1720,7 @@
         <v>2023</v>
       </c>
     </row>
-    <row r="59" spans="1:5">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
         <v>47</v>
       </c>
@@ -1689,7 +1734,7 @@
         <v>2023</v>
       </c>
     </row>
-    <row r="60" spans="1:5">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
         <v>48</v>
       </c>
@@ -1703,7 +1748,7 @@
         <v>2023</v>
       </c>
     </row>
-    <row r="61" spans="1:5">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
         <v>49</v>
       </c>
@@ -1717,7 +1762,7 @@
         <v>2023</v>
       </c>
     </row>
-    <row r="62" spans="1:5">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
         <v>50</v>
       </c>
@@ -1731,7 +1776,7 @@
         <v>2023</v>
       </c>
     </row>
-    <row r="63" spans="1:5">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
         <v>51</v>
       </c>
@@ -1745,7 +1790,7 @@
         <v>2023</v>
       </c>
     </row>
-    <row r="64" spans="1:5">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
         <v>52</v>
       </c>
@@ -1759,7 +1804,7 @@
         <v>2023</v>
       </c>
     </row>
-    <row r="65" spans="1:5">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
         <v>53</v>
       </c>
@@ -1773,7 +1818,7 @@
         <v>2023</v>
       </c>
     </row>
-    <row r="66" spans="1:5">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
         <v>54</v>
       </c>
@@ -1787,7 +1832,7 @@
         <v>2023</v>
       </c>
     </row>
-    <row r="67" spans="1:5">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
         <v>69</v>
       </c>
@@ -1804,7 +1849,7 @@
         <v>2024</v>
       </c>
     </row>
-    <row r="68" spans="1:5">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
         <v>70</v>
       </c>
@@ -1821,7 +1866,7 @@
         <v>2024</v>
       </c>
     </row>
-    <row r="69" spans="1:5">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
         <v>71</v>
       </c>
@@ -1838,7 +1883,7 @@
         <v>2024</v>
       </c>
     </row>
-    <row r="70" spans="1:5">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
         <v>72</v>
       </c>
@@ -1855,7 +1900,7 @@
         <v>2024</v>
       </c>
     </row>
-    <row r="71" spans="1:5">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" s="1" t="s">
         <v>73</v>
       </c>
@@ -1872,21 +1917,174 @@
         <v>2024</v>
       </c>
     </row>
-    <row r="72" spans="1:5">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" s="1" t="s">
-        <v>83</v>
+        <v>147</v>
       </c>
       <c r="B72" t="s">
-        <v>84</v>
+        <v>148</v>
       </c>
       <c r="C72" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="D72" s="1" t="s">
         <v>86</v>
       </c>
       <c r="E72">
         <v>2025</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A73" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="B73" t="s">
+        <v>84</v>
+      </c>
+      <c r="C73" t="s">
+        <v>85</v>
+      </c>
+      <c r="D73" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="E73">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A74" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="B74" t="s">
+        <v>146</v>
+      </c>
+      <c r="C74" t="s">
+        <v>81</v>
+      </c>
+      <c r="D74" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="E74">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A75" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="B75" t="s">
+        <v>78</v>
+      </c>
+      <c r="C75" t="s">
+        <v>79</v>
+      </c>
+      <c r="D75" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="E75">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A76" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="B76" t="s">
+        <v>151</v>
+      </c>
+      <c r="C76" t="s">
+        <v>82</v>
+      </c>
+      <c r="D76" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="E76">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A77" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="B77" t="s">
+        <v>148</v>
+      </c>
+      <c r="C77" t="s">
+        <v>80</v>
+      </c>
+      <c r="D77" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="E77">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A78" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="B78" t="s">
+        <v>84</v>
+      </c>
+      <c r="C78" t="s">
+        <v>85</v>
+      </c>
+      <c r="D78" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="E78">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A79" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="B79" t="s">
+        <v>78</v>
+      </c>
+      <c r="C79" t="s">
+        <v>79</v>
+      </c>
+      <c r="D79" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="E79">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A80" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="B80" t="s">
+        <v>151</v>
+      </c>
+      <c r="C80" t="s">
+        <v>82</v>
+      </c>
+      <c r="D80" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="E80">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A81" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="B81" t="s">
+        <v>158</v>
+      </c>
+      <c r="C81" t="s">
+        <v>159</v>
+      </c>
+      <c r="D81" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="E81">
+        <v>2026</v>
       </c>
     </row>
   </sheetData>

</xml_diff>